<commit_message>
fix(checkout): gestione flessibile destinazione tomba/funerale per piante in vaso senza obbligo data funerale [FLOREM_AUTO_PROT]
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/verbali/FloreMoria_2026_T1_Corrispettivi.xlsx
+++ b/docs/verbali/FloreMoria_2026_T1_Corrispettivi.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="69">
   <si>
     <t>Ragione sociale</t>
   </si>
@@ -35,7 +35,7 @@
     <t>Data e ora generazione</t>
   </si>
   <si>
-    <t>20/09/2026, 19:23:44</t>
+    <t>21/09/2026, 22:23:47</t>
   </si>
   <si>
     <t>Voce</t>
@@ -80,13 +80,7 @@
     <t>Nota 3</t>
   </si>
   <si>
-    <t>Foglio F3 (costi fiorista senza documento) sospeso: rientrerà quando l’abbinamento bonifici→consegne sarà corretto. Non usare i movimenti bancari come proxy del costo per consegna.</t>
-  </si>
-  <si>
-    <t>Nota 4</t>
-  </si>
-  <si>
-    <t>Prima di chiudere il trimestre caricare l’estratto conto Fineco aggiornato in Contabilità → Movimenti bancari.</t>
+    <t>I costi verso i fioristi sono comunicati separatamente.</t>
   </si>
   <si>
     <t>Data ordine</t>
@@ -101,22 +95,138 @@
     <t>IVA EUR</t>
   </si>
   <si>
-    <t>DA_COLLEGARE</t>
+    <t>16/01/2026</t>
+  </si>
+  <si>
+    <t>66C04847WL650301D</t>
   </si>
   <si>
     <t>PayPal</t>
   </si>
   <si>
+    <t>20/01/2026</t>
+  </si>
+  <si>
+    <t>ch_3Src7YRrkwwcYwep0jrAiVTa</t>
+  </si>
+  <si>
     <t>Stripe</t>
+  </si>
+  <si>
+    <t>21/01/2026</t>
+  </si>
+  <si>
+    <t>22E30531F99808504</t>
+  </si>
+  <si>
+    <t>22/01/2026</t>
+  </si>
+  <si>
+    <t>8YH43677SS377553L</t>
+  </si>
+  <si>
+    <t>ch_3SsPVeRrkwwcYwep18ol6Ovs</t>
+  </si>
+  <si>
+    <t>09/02/2026</t>
+  </si>
+  <si>
+    <t>44E519039S467634K</t>
+  </si>
+  <si>
+    <t>16/02/2026</t>
+  </si>
+  <si>
+    <t>2GU64478W4726692S</t>
+  </si>
+  <si>
+    <t>19/02/2026</t>
+  </si>
+  <si>
+    <t>ch_3T2SsURrkwwcYwep02GfXa8W</t>
+  </si>
+  <si>
+    <t>22/02/2026</t>
+  </si>
+  <si>
+    <t>4W6628604D401674M</t>
+  </si>
+  <si>
+    <t>25/02/2026</t>
+  </si>
+  <si>
+    <t>ch_3T4dUERrkwwcYwep12Oam9Z2</t>
+  </si>
+  <si>
+    <t>26/02/2026</t>
+  </si>
+  <si>
+    <t>ch_3T4uOsRrkwwcYwep1zRSm9BF</t>
+  </si>
+  <si>
+    <t>01/03/2026</t>
+  </si>
+  <si>
+    <t>ch_3T6AndRrkwwcYwep0qzntmsz</t>
+  </si>
+  <si>
+    <t>13/03/2026</t>
+  </si>
+  <si>
+    <t>83N54580AU0027713</t>
+  </si>
+  <si>
+    <t>14/03/2026</t>
+  </si>
+  <si>
+    <t>3D552868PU399581S</t>
+  </si>
+  <si>
+    <t>ch_3TArJQRrkwwcYwep1euDxquO</t>
+  </si>
+  <si>
+    <t>18/03/2026</t>
+  </si>
+  <si>
+    <t>ch_3TCJsERrkwwcYwep0iZJueLR</t>
+  </si>
+  <si>
+    <t>19/03/2026</t>
+  </si>
+  <si>
+    <t>ch_3TCgrURrkwwcYwep0MNWC4e8</t>
+  </si>
+  <si>
+    <t>22/03/2026</t>
+  </si>
+  <si>
+    <t>95E92452N40245344</t>
+  </si>
+  <si>
+    <t>24/03/2026</t>
+  </si>
+  <si>
+    <t>09C2701554000764W</t>
+  </si>
+  <si>
+    <t>29/03/2026</t>
+  </si>
+  <si>
+    <t>ch_3TG8URRrkwwcYwep12OHecA0</t>
+  </si>
+  <si>
+    <t>31/03/2026</t>
+  </si>
+  <si>
+    <t>ch_3TH2KrRrkwwcYwep1njcWN9l</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="€ #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -182,7 +292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -192,7 +302,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,7 +641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -660,14 +769,6 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" t="s">
-        <v>24</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -679,8 +780,8 @@
   <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="29" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="6" width="12" customWidth="1"/>
@@ -689,13 +790,13 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>10</v>
@@ -704,21 +805,21 @@
         <v>11</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="7">
-        <v>46038.45833333333</v>
+      <c r="A2" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D2" s="3">
         <v>36.35</v>
@@ -734,14 +835,14 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="7">
-        <v>46042.45833333333</v>
+      <c r="A3" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D3" s="3">
         <v>36.35</v>
@@ -757,14 +858,14 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="7">
-        <v>46043.45833333333</v>
+      <c r="A4" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D4" s="3">
         <v>27.26</v>
@@ -780,14 +881,14 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
-        <v>46044.45833333333</v>
+      <c r="A5" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D5" s="3">
         <v>27.26</v>
@@ -803,14 +904,14 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
-        <v>46044.45833333333</v>
+      <c r="A6" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" s="3">
         <v>37.25</v>
@@ -826,14 +927,14 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
-        <v>46062.45833333333</v>
+      <c r="A7" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D7" s="3">
         <v>36.35</v>
@@ -849,14 +950,14 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
-        <v>46069.45833333333</v>
+      <c r="A8" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D8" s="3">
         <v>27.26</v>
@@ -872,14 +973,14 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
-        <v>46072.45833333333</v>
+      <c r="A9" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D9" s="3">
         <v>36.35</v>
@@ -895,14 +996,14 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
-        <v>46075.45833333333</v>
+      <c r="A10" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D10" s="3">
         <v>27.26</v>
@@ -918,14 +1019,14 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
-        <v>46078.45833333333</v>
+      <c r="A11" s="2" t="s">
+        <v>46</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D11" s="3">
         <v>27.26</v>
@@ -941,14 +1042,14 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="7">
-        <v>46079.45833333333</v>
+      <c r="A12" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D12" s="3">
         <v>36.35</v>
@@ -964,14 +1065,14 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="7">
-        <v>46082.45833333333</v>
+      <c r="A13" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D13" s="3">
         <v>131.8</v>
@@ -987,14 +1088,14 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="7">
-        <v>46094.45833333333</v>
+      <c r="A14" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D14" s="3">
         <v>45.45</v>
@@ -1010,14 +1111,14 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="7">
-        <v>46095.45833333333</v>
+      <c r="A15" s="2" t="s">
+        <v>54</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D15" s="3">
         <v>65.89</v>
@@ -1033,14 +1134,14 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="7">
-        <v>46095.45833333333</v>
+      <c r="A16" s="2" t="s">
+        <v>54</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D16" s="3">
         <v>63.62</v>
@@ -1056,14 +1157,14 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="7">
-        <v>46099.45833333333</v>
+      <c r="A17" s="2" t="s">
+        <v>57</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D17" s="3">
         <v>36.35</v>
@@ -1079,14 +1180,14 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="7">
-        <v>46100.45833333333</v>
+      <c r="A18" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D18" s="3">
         <v>31.81</v>
@@ -1102,14 +1203,14 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="7">
-        <v>46103.45833333333</v>
+      <c r="A19" s="2" t="s">
+        <v>61</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D19" s="3">
         <v>27.26</v>
@@ -1125,14 +1226,14 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="7">
-        <v>46105.45833333333</v>
+      <c r="A20" s="2" t="s">
+        <v>63</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D20" s="3">
         <v>27.26</v>
@@ -1148,14 +1249,14 @@
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="7">
-        <v>46110.41666666667</v>
+      <c r="A21" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D21" s="3">
         <v>27.26</v>
@@ -1171,14 +1272,14 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="7">
-        <v>46112.41666666667</v>
+      <c r="A22" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D22" s="3">
         <v>131.8</v>

</xml_diff>